<commit_message>
Refine template UX and preserve source form geometry
</commit_message>
<xml_diff>
--- a/assets/templates/commercial-invoice.xlsx
+++ b/assets/templates/commercial-invoice.xlsx
@@ -7,7 +7,7 @@
     <sheet sheetId="1" name="CI" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'CI'!$A1:$I78</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'CI'!$A1:$K50</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
@@ -76,7 +76,7 @@
     <t>TOTAL QUANTITY :</t>
   </si>
   <si>
-    <t>TOTAL AMOUT :</t>
+    <t>TOTAL AMOUNT :</t>
   </si>
   <si>
     <t>Signed by</t>
@@ -167,7 +167,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -179,9 +179,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -526,17 +523,19 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I78"/>
+  <dimension ref="A1:K50"/>
   <sheetFormatPr defaultRowHeight="18" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="3" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="10" customWidth="1"/>
-    <col min="7" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="1" max="1" width="10.17" customWidth="1"/>
+    <col min="2" max="2" width="9.92" customWidth="1"/>
+    <col min="3" max="3" width="11.17" customWidth="1"/>
+    <col min="4" max="4" width="15.67" customWidth="1"/>
+    <col min="5" max="5" width="8.58" customWidth="1"/>
+    <col min="6" max="6" width="7.17" customWidth="1"/>
+    <col min="7" max="7" width="9.83" customWidth="1"/>
+    <col min="8" max="8" width="13.42" customWidth="1"/>
+    <col min="9" max="9" width="10.58" customWidth="1"/>
+    <col min="10" max="11" width="10" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -760,443 +759,334 @@
         <v>18</v>
       </c>
     </row>
-    <row r="23" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" ht="23" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="3"/>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
       <c r="D23" s="3"/>
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
-    </row>
-    <row r="24" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="3"/>
+      <c r="J23" s="3"/>
+      <c r="K23" s="3"/>
+    </row>
+    <row r="24" ht="23" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
       <c r="D24" s="3"/>
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
-    </row>
-    <row r="25" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="3"/>
+      <c r="K24" s="3"/>
+    </row>
+    <row r="25" ht="23" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="3"/>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
-    </row>
-    <row r="26" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="3"/>
+      <c r="K25" s="3"/>
+    </row>
+    <row r="26" ht="23" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="3"/>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
-    </row>
-    <row r="27" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+      <c r="I26" s="3"/>
+      <c r="J26" s="3"/>
+      <c r="K26" s="3"/>
+    </row>
+    <row r="27" ht="23" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="3"/>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
-    </row>
-    <row r="28" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
+      <c r="I27" s="3"/>
+      <c r="J27" s="3"/>
+      <c r="K27" s="3"/>
+    </row>
+    <row r="28" ht="23" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="3"/>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
-    </row>
-    <row r="29" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="3"/>
+      <c r="J28" s="3"/>
+      <c r="K28" s="3"/>
+    </row>
+    <row r="29" ht="23" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="3"/>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
       <c r="E29" s="3"/>
       <c r="F29" s="3"/>
-    </row>
-    <row r="30" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G29" s="3"/>
+      <c r="H29" s="3"/>
+      <c r="I29" s="3"/>
+      <c r="J29" s="3"/>
+      <c r="K29" s="3"/>
+    </row>
+    <row r="30" ht="23" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>
       <c r="E30" s="3"/>
       <c r="F30" s="3"/>
-    </row>
-    <row r="31" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G30" s="3"/>
+      <c r="H30" s="3"/>
+      <c r="I30" s="3"/>
+      <c r="J30" s="3"/>
+      <c r="K30" s="3"/>
+    </row>
+    <row r="31" ht="23" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
       <c r="D31" s="3"/>
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
-    </row>
-    <row r="32" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G31" s="3"/>
+      <c r="H31" s="3"/>
+      <c r="I31" s="3"/>
+      <c r="J31" s="3"/>
+      <c r="K31" s="3"/>
+    </row>
+    <row r="32" ht="23" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
-    </row>
-    <row r="33" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G32" s="3"/>
+      <c r="H32" s="3"/>
+      <c r="I32" s="3"/>
+      <c r="J32" s="3"/>
+      <c r="K32" s="3"/>
+    </row>
+    <row r="33" ht="23" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="3"/>
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
       <c r="D33" s="3"/>
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
-    </row>
-    <row r="34" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G33" s="3"/>
+      <c r="H33" s="3"/>
+      <c r="I33" s="3"/>
+      <c r="J33" s="3"/>
+      <c r="K33" s="3"/>
+    </row>
+    <row r="34" ht="23" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="3"/>
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
       <c r="D34" s="3"/>
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
-    </row>
-    <row r="35" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G34" s="3"/>
+      <c r="H34" s="3"/>
+      <c r="I34" s="3"/>
+      <c r="J34" s="3"/>
+      <c r="K34" s="3"/>
+    </row>
+    <row r="35" ht="23" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="3"/>
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
       <c r="D35" s="3"/>
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
-    </row>
-    <row r="36" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G35" s="3"/>
+      <c r="H35" s="3"/>
+      <c r="I35" s="3"/>
+      <c r="J35" s="3"/>
+      <c r="K35" s="3"/>
+    </row>
+    <row r="36" ht="23" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="3"/>
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
-    </row>
-    <row r="37" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G36" s="3"/>
+      <c r="H36" s="3"/>
+      <c r="I36" s="3"/>
+      <c r="J36" s="3"/>
+      <c r="K36" s="3"/>
+    </row>
+    <row r="37" ht="23" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="3"/>
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
       <c r="D37" s="3"/>
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
-    </row>
-    <row r="38" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G37" s="3"/>
+      <c r="H37" s="3"/>
+      <c r="I37" s="3"/>
+      <c r="J37" s="3"/>
+      <c r="K37" s="3"/>
+    </row>
+    <row r="38" ht="23" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="3"/>
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
       <c r="D38" s="3"/>
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
-    </row>
-    <row r="39" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G38" s="3"/>
+      <c r="H38" s="3"/>
+      <c r="I38" s="3"/>
+      <c r="J38" s="3"/>
+      <c r="K38" s="3"/>
+    </row>
+    <row r="39" ht="23" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="3"/>
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
       <c r="E39" s="3"/>
       <c r="F39" s="3"/>
-    </row>
-    <row r="40" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G39" s="3"/>
+      <c r="H39" s="3"/>
+      <c r="I39" s="3"/>
+      <c r="J39" s="3"/>
+      <c r="K39" s="3"/>
+    </row>
+    <row r="40" ht="23" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="3"/>
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
       <c r="D40" s="3"/>
       <c r="E40" s="3"/>
       <c r="F40" s="3"/>
-    </row>
-    <row r="41" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G40" s="3"/>
+      <c r="H40" s="3"/>
+      <c r="I40" s="3"/>
+      <c r="J40" s="3"/>
+      <c r="K40" s="3"/>
+    </row>
+    <row r="41" ht="23" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="3"/>
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
       <c r="D41" s="3"/>
       <c r="E41" s="3"/>
       <c r="F41" s="3"/>
-    </row>
-    <row r="42" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G41" s="3"/>
+      <c r="H41" s="3"/>
+      <c r="I41" s="3"/>
+      <c r="J41" s="3"/>
+      <c r="K41" s="3"/>
+    </row>
+    <row r="42" ht="23" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="3"/>
       <c r="B42" s="3"/>
       <c r="C42" s="3"/>
       <c r="D42" s="3"/>
       <c r="E42" s="3"/>
       <c r="F42" s="3"/>
-    </row>
-    <row r="43" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G42" s="3"/>
+      <c r="H42" s="3"/>
+      <c r="I42" s="3"/>
+      <c r="J42" s="3"/>
+      <c r="K42" s="3"/>
+    </row>
+    <row r="43" ht="23" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="3"/>
       <c r="B43" s="3"/>
       <c r="C43" s="3"/>
       <c r="D43" s="3"/>
       <c r="E43" s="3"/>
       <c r="F43" s="3"/>
-    </row>
-    <row r="44" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G43" s="3"/>
+      <c r="H43" s="3"/>
+      <c r="I43" s="3"/>
+      <c r="J43" s="3"/>
+      <c r="K43" s="3"/>
+    </row>
+    <row r="44" ht="23" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" s="3"/>
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
       <c r="D44" s="3"/>
       <c r="E44" s="3"/>
       <c r="F44" s="3"/>
-    </row>
-    <row r="45" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G44" s="3"/>
+      <c r="H44" s="3"/>
+      <c r="I44" s="3"/>
+      <c r="J44" s="3"/>
+      <c r="K44" s="3"/>
+    </row>
+    <row r="45" ht="23" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="3"/>
       <c r="B45" s="3"/>
       <c r="C45" s="3"/>
       <c r="D45" s="3"/>
       <c r="E45" s="3"/>
       <c r="F45" s="3"/>
-    </row>
-    <row r="46" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A46" s="3"/>
-      <c r="B46" s="3"/>
-      <c r="C46" s="3"/>
-      <c r="D46" s="3"/>
-      <c r="E46" s="3"/>
-      <c r="F46" s="3"/>
-    </row>
-    <row r="47" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A47" s="3"/>
-      <c r="B47" s="3"/>
-      <c r="C47" s="3"/>
-      <c r="D47" s="3"/>
-      <c r="E47" s="3"/>
-      <c r="F47" s="3"/>
-    </row>
-    <row r="48" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A48" s="3"/>
-      <c r="B48" s="3"/>
-      <c r="C48" s="3"/>
-      <c r="D48" s="3"/>
-      <c r="E48" s="3"/>
-      <c r="F48" s="3"/>
-    </row>
-    <row r="49" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A49" s="3"/>
-      <c r="B49" s="3"/>
-      <c r="C49" s="3"/>
-      <c r="D49" s="3"/>
-      <c r="E49" s="3"/>
-      <c r="F49" s="3"/>
-    </row>
-    <row r="50" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A50" s="3"/>
-      <c r="B50" s="3"/>
-      <c r="C50" s="3"/>
-      <c r="D50" s="3"/>
-      <c r="E50" s="3"/>
+      <c r="G45" s="3"/>
+      <c r="H45" s="3"/>
+      <c r="I45" s="3"/>
+      <c r="J45" s="3"/>
+      <c r="K45" s="3"/>
+    </row>
+    <row r="46" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E46" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="47" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E47" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="49" spans="6:9" x14ac:dyDescent="0.25">
+      <c r="F49" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="G49" s="3"/>
+      <c r="H49" s="3"/>
+      <c r="I49" s="3"/>
+    </row>
+    <row r="50" spans="5:9" x14ac:dyDescent="0.25">
+      <c r="E50" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="F50" s="3"/>
-    </row>
-    <row r="51" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A51" s="3"/>
-      <c r="B51" s="3"/>
-      <c r="C51" s="3"/>
-      <c r="D51" s="3"/>
-      <c r="E51" s="3"/>
-      <c r="F51" s="3"/>
-    </row>
-    <row r="52" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A52" s="3"/>
-      <c r="B52" s="3"/>
-      <c r="C52" s="3"/>
-      <c r="D52" s="3"/>
-      <c r="E52" s="3"/>
-      <c r="F52" s="3"/>
-    </row>
-    <row r="53" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A53" s="3"/>
-      <c r="B53" s="3"/>
-      <c r="C53" s="3"/>
-      <c r="D53" s="3"/>
-      <c r="E53" s="3"/>
-      <c r="F53" s="3"/>
-    </row>
-    <row r="54" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A54" s="3"/>
-      <c r="B54" s="3"/>
-      <c r="C54" s="3"/>
-      <c r="D54" s="3"/>
-      <c r="E54" s="3"/>
-      <c r="F54" s="3"/>
-    </row>
-    <row r="55" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A55" s="3"/>
-      <c r="B55" s="3"/>
-      <c r="C55" s="3"/>
-      <c r="D55" s="3"/>
-      <c r="E55" s="3"/>
-      <c r="F55" s="3"/>
-    </row>
-    <row r="56" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A56" s="3"/>
-      <c r="B56" s="3"/>
-      <c r="C56" s="3"/>
-      <c r="D56" s="3"/>
-      <c r="E56" s="3"/>
-      <c r="F56" s="3"/>
-    </row>
-    <row r="57" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A57" s="3"/>
-      <c r="B57" s="3"/>
-      <c r="C57" s="3"/>
-      <c r="D57" s="3"/>
-      <c r="E57" s="3"/>
-      <c r="F57" s="3"/>
-    </row>
-    <row r="58" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A58" s="3"/>
-      <c r="B58" s="3"/>
-      <c r="C58" s="3"/>
-      <c r="D58" s="3"/>
-      <c r="E58" s="3"/>
-      <c r="F58" s="3"/>
-    </row>
-    <row r="59" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A59" s="3"/>
-      <c r="B59" s="3"/>
-      <c r="C59" s="3"/>
-      <c r="D59" s="3"/>
-      <c r="E59" s="3"/>
-      <c r="F59" s="3"/>
-    </row>
-    <row r="60" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A60" s="3"/>
-      <c r="B60" s="3"/>
-      <c r="C60" s="3"/>
-      <c r="D60" s="3"/>
-      <c r="E60" s="3"/>
-      <c r="F60" s="3"/>
-    </row>
-    <row r="61" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A61" s="3"/>
-      <c r="B61" s="3"/>
-      <c r="C61" s="3"/>
-      <c r="D61" s="3"/>
-      <c r="E61" s="3"/>
-      <c r="F61" s="3"/>
-    </row>
-    <row r="62" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A62" s="3"/>
-      <c r="B62" s="3"/>
-      <c r="C62" s="3"/>
-      <c r="D62" s="3"/>
-      <c r="E62" s="3"/>
-      <c r="F62" s="3"/>
-    </row>
-    <row r="63" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A63" s="3"/>
-      <c r="B63" s="3"/>
-      <c r="C63" s="3"/>
-      <c r="D63" s="3"/>
-      <c r="E63" s="3"/>
-      <c r="F63" s="3"/>
-    </row>
-    <row r="64" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A64" s="3"/>
-      <c r="B64" s="3"/>
-      <c r="C64" s="3"/>
-      <c r="D64" s="3"/>
-      <c r="E64" s="3"/>
-      <c r="F64" s="3"/>
-    </row>
-    <row r="65" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A65" s="3"/>
-      <c r="B65" s="3"/>
-      <c r="C65" s="3"/>
-      <c r="D65" s="3"/>
-      <c r="E65" s="3"/>
-      <c r="F65" s="3"/>
-    </row>
-    <row r="66" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A66" s="3"/>
-      <c r="B66" s="3"/>
-      <c r="C66" s="3"/>
-      <c r="D66" s="3"/>
-      <c r="E66" s="3"/>
-      <c r="F66" s="3"/>
-    </row>
-    <row r="67" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A67" s="3"/>
-      <c r="B67" s="3"/>
-      <c r="C67" s="3"/>
-      <c r="D67" s="3"/>
-      <c r="E67" s="3"/>
-      <c r="F67" s="3"/>
-    </row>
-    <row r="68" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A68" s="3"/>
-      <c r="B68" s="3"/>
-      <c r="C68" s="3"/>
-      <c r="D68" s="3"/>
-      <c r="E68" s="3"/>
-      <c r="F68" s="3"/>
-    </row>
-    <row r="69" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A69" s="3"/>
-      <c r="B69" s="3"/>
-      <c r="C69" s="3"/>
-      <c r="D69" s="3"/>
-      <c r="E69" s="3"/>
-      <c r="F69" s="3"/>
-    </row>
-    <row r="70" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A70" s="3"/>
-      <c r="B70" s="3"/>
-      <c r="C70" s="3"/>
-      <c r="D70" s="3"/>
-      <c r="E70" s="3"/>
-      <c r="F70" s="3"/>
-    </row>
-    <row r="71" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A71" s="3"/>
-      <c r="B71" s="3"/>
-      <c r="C71" s="3"/>
-      <c r="D71" s="3"/>
-      <c r="E71" s="3"/>
-      <c r="F71" s="3"/>
-    </row>
-    <row r="72" ht="23" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A72" s="3"/>
-      <c r="B72" s="3"/>
-      <c r="C72" s="3"/>
-      <c r="D72" s="3"/>
-      <c r="E72" s="3"/>
-      <c r="F72" s="3"/>
-    </row>
-    <row r="74" spans="5:9" x14ac:dyDescent="0.25">
-      <c r="E74" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="F74" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I74" s="3"/>
-    </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A77" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B77" s="2"/>
-      <c r="C77" s="2"/>
-      <c r="D77" s="2"/>
-      <c r="E77" s="2"/>
-      <c r="F77" s="2"/>
-      <c r="G77" s="2"/>
-      <c r="H77" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="I77" s="3"/>
-    </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A78" s="2"/>
-      <c r="B78" s="2"/>
-      <c r="C78" s="2"/>
-      <c r="D78" s="2"/>
-      <c r="E78" s="2"/>
-      <c r="F78" s="2"/>
-      <c r="G78" s="2"/>
-      <c r="H78" s="3"/>
-      <c r="I78" s="3"/>
+      <c r="G50" s="3"/>
+      <c r="H50" s="3"/>
+      <c r="I50" s="3"/>
     </row>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="22">
     <mergeCell ref="A1:I2"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="E4:G4"/>
@@ -1218,8 +1108,7 @@
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="C21:D21"/>
     <mergeCell ref="E21:I21"/>
-    <mergeCell ref="A77:G78"/>
-    <mergeCell ref="H77:I78"/>
+    <mergeCell ref="F49:I50"/>
   </mergeCells>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>